<commit_message>
fix(legal-os): simplify review gates and correct draft amount handling
</commit_message>
<xml_diff>
--- a/skills/legal-os-data-verification/assets/templates/Legal_OS_v1.7_Amount_Data_Verification_Workspace.xlsx
+++ b/skills/legal-os-data-verification/assets/templates/Legal_OS_v1.7_Amount_Data_Verification_Workspace.xlsx
@@ -878,6 +878,17 @@
     <x:col min="11" max="11" width="16" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="12" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="24" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="14" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="18" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="24" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="28" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="15" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="18" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="32" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="10" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="16" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="30" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="20" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -890,6 +901,11 @@
         <x:v>只抄录可由来源文件、凭证或经确认的记录直接支持的值。三行 DEMO 数据可删除后替换。</x:v>
       </x:c>
     </x:row>
+    <x:row r="3" ht="34" customHeight="1">
+      <x:c r="A3" s="8" t="str">
+        <x:v>金额链一次录入：原值J、已付K直接引用；扩展列N:X描述链条。固定扣减/抵扣复用J，付款复用K；原行K&gt;0须另填W:X付款凭证。</x:v>
+      </x:c>
+    </x:row>
     <x:row r="4" ht="28" customHeight="1">
       <x:c r="A4" s="14" t="str">
         <x:v>记录ID</x:v>
@@ -930,6 +946,39 @@
       <x:c r="M4" s="14" t="str">
         <x:v>备注</x:v>
       </x:c>
+      <x:c r="N4" s="14" t="str">
+        <x:v>链条ID</x:v>
+      </x:c>
+      <x:c r="O4" s="14" t="str">
+        <x:v>记录类型</x:v>
+      </x:c>
+      <x:c r="P4" s="14" t="str">
+        <x:v>因素ID</x:v>
+      </x:c>
+      <x:c r="Q4" s="14" t="str">
+        <x:v>计算依据（上一步记录ID）</x:v>
+      </x:c>
+      <x:c r="R4" s="14" t="str">
+        <x:v>因素类型</x:v>
+      </x:c>
+      <x:c r="S4" s="14" t="str">
+        <x:v>因素值（百分率小数）</x:v>
+      </x:c>
+      <x:c r="T4" s="14" t="str">
+        <x:v>原金额已含因素ID（分号分隔）</x:v>
+      </x:c>
+      <x:c r="U4" s="14" t="str">
+        <x:v>小数位</x:v>
+      </x:c>
+      <x:c r="V4" s="14" t="str">
+        <x:v>舍入规则</x:v>
+      </x:c>
+      <x:c r="W4" s="14" t="str">
+        <x:v>付款来源定位（原行K&gt;0时）</x:v>
+      </x:c>
+      <x:c r="X4" s="14" t="str">
+        <x:v>付款证据状态（原行K&gt;0时）</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="28" t="str">
@@ -971,6 +1020,17 @@
       <x:c r="M5" s="29" t="str">
         <x:v>演示数据：可删除</x:v>
       </x:c>
+      <x:c r="N5" s="34"/>
+      <x:c r="O5" s="34"/>
+      <x:c r="P5" s="34"/>
+      <x:c r="Q5" s="34"/>
+      <x:c r="R5" s="34"/>
+      <x:c r="S5" s="34"/>
+      <x:c r="T5" s="34"/>
+      <x:c r="U5" s="34"/>
+      <x:c r="V5" s="34"/>
+      <x:c r="W5" s="34"/>
+      <x:c r="X5" s="34"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="30" t="str">
@@ -1012,6 +1072,17 @@
       <x:c r="M6" s="31" t="str">
         <x:v>演示数据：证据待核</x:v>
       </x:c>
+      <x:c r="N6" s="36"/>
+      <x:c r="O6" s="36"/>
+      <x:c r="P6" s="36"/>
+      <x:c r="Q6" s="36"/>
+      <x:c r="R6" s="36"/>
+      <x:c r="S6" s="36"/>
+      <x:c r="T6" s="36"/>
+      <x:c r="U6" s="36"/>
+      <x:c r="V6" s="36"/>
+      <x:c r="W6" s="36"/>
+      <x:c r="X6" s="36"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="30" t="str">
@@ -1053,6 +1124,17 @@
       <x:c r="M7" s="31" t="str">
         <x:v>演示数据：可删除</x:v>
       </x:c>
+      <x:c r="N7" s="34"/>
+      <x:c r="O7" s="34"/>
+      <x:c r="P7" s="34"/>
+      <x:c r="Q7" s="34"/>
+      <x:c r="R7" s="34"/>
+      <x:c r="S7" s="34"/>
+      <x:c r="T7" s="34"/>
+      <x:c r="U7" s="34"/>
+      <x:c r="V7" s="34"/>
+      <x:c r="W7" s="34"/>
+      <x:c r="X7" s="34"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="30"/>
@@ -1068,6 +1150,17 @@
       <x:c r="K8" s="52"/>
       <x:c r="L8" s="36"/>
       <x:c r="M8" s="31"/>
+      <x:c r="N8" s="36"/>
+      <x:c r="O8" s="36"/>
+      <x:c r="P8" s="36"/>
+      <x:c r="Q8" s="36"/>
+      <x:c r="R8" s="36"/>
+      <x:c r="S8" s="36"/>
+      <x:c r="T8" s="36"/>
+      <x:c r="U8" s="36"/>
+      <x:c r="V8" s="36"/>
+      <x:c r="W8" s="36"/>
+      <x:c r="X8" s="36"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="30"/>
@@ -1083,6 +1176,17 @@
       <x:c r="K9" s="52"/>
       <x:c r="L9" s="36"/>
       <x:c r="M9" s="31"/>
+      <x:c r="N9" s="34"/>
+      <x:c r="O9" s="34"/>
+      <x:c r="P9" s="34"/>
+      <x:c r="Q9" s="34"/>
+      <x:c r="R9" s="34"/>
+      <x:c r="S9" s="34"/>
+      <x:c r="T9" s="34"/>
+      <x:c r="U9" s="34"/>
+      <x:c r="V9" s="34"/>
+      <x:c r="W9" s="34"/>
+      <x:c r="X9" s="34"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="30"/>
@@ -1098,6 +1202,17 @@
       <x:c r="K10" s="52"/>
       <x:c r="L10" s="36"/>
       <x:c r="M10" s="31"/>
+      <x:c r="N10" s="36"/>
+      <x:c r="O10" s="36"/>
+      <x:c r="P10" s="36"/>
+      <x:c r="Q10" s="36"/>
+      <x:c r="R10" s="36"/>
+      <x:c r="S10" s="36"/>
+      <x:c r="T10" s="36"/>
+      <x:c r="U10" s="36"/>
+      <x:c r="V10" s="36"/>
+      <x:c r="W10" s="36"/>
+      <x:c r="X10" s="36"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="30"/>
@@ -1113,6 +1228,17 @@
       <x:c r="K11" s="52"/>
       <x:c r="L11" s="36"/>
       <x:c r="M11" s="31"/>
+      <x:c r="N11" s="34"/>
+      <x:c r="O11" s="34"/>
+      <x:c r="P11" s="34"/>
+      <x:c r="Q11" s="34"/>
+      <x:c r="R11" s="34"/>
+      <x:c r="S11" s="34"/>
+      <x:c r="T11" s="34"/>
+      <x:c r="U11" s="34"/>
+      <x:c r="V11" s="34"/>
+      <x:c r="W11" s="34"/>
+      <x:c r="X11" s="34"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="30"/>
@@ -1128,6 +1254,17 @@
       <x:c r="K12" s="52"/>
       <x:c r="L12" s="36"/>
       <x:c r="M12" s="31"/>
+      <x:c r="N12" s="36"/>
+      <x:c r="O12" s="36"/>
+      <x:c r="P12" s="36"/>
+      <x:c r="Q12" s="36"/>
+      <x:c r="R12" s="36"/>
+      <x:c r="S12" s="36"/>
+      <x:c r="T12" s="36"/>
+      <x:c r="U12" s="36"/>
+      <x:c r="V12" s="36"/>
+      <x:c r="W12" s="36"/>
+      <x:c r="X12" s="36"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="30"/>
@@ -1143,6 +1280,17 @@
       <x:c r="K13" s="52"/>
       <x:c r="L13" s="36"/>
       <x:c r="M13" s="31"/>
+      <x:c r="N13" s="34"/>
+      <x:c r="O13" s="34"/>
+      <x:c r="P13" s="34"/>
+      <x:c r="Q13" s="34"/>
+      <x:c r="R13" s="34"/>
+      <x:c r="S13" s="34"/>
+      <x:c r="T13" s="34"/>
+      <x:c r="U13" s="34"/>
+      <x:c r="V13" s="34"/>
+      <x:c r="W13" s="34"/>
+      <x:c r="X13" s="34"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="30"/>
@@ -1158,6 +1306,17 @@
       <x:c r="K14" s="52"/>
       <x:c r="L14" s="36"/>
       <x:c r="M14" s="31"/>
+      <x:c r="N14" s="36"/>
+      <x:c r="O14" s="36"/>
+      <x:c r="P14" s="36"/>
+      <x:c r="Q14" s="36"/>
+      <x:c r="R14" s="36"/>
+      <x:c r="S14" s="36"/>
+      <x:c r="T14" s="36"/>
+      <x:c r="U14" s="36"/>
+      <x:c r="V14" s="36"/>
+      <x:c r="W14" s="36"/>
+      <x:c r="X14" s="36"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="32"/>
@@ -1173,11 +1332,22 @@
       <x:c r="K15" s="53"/>
       <x:c r="L15" s="47"/>
       <x:c r="M15" s="33"/>
+      <x:c r="N15" s="34"/>
+      <x:c r="O15" s="34"/>
+      <x:c r="P15" s="34"/>
+      <x:c r="Q15" s="34"/>
+      <x:c r="R15" s="34"/>
+      <x:c r="S15" s="34"/>
+      <x:c r="T15" s="34"/>
+      <x:c r="U15" s="34"/>
+      <x:c r="V15" s="34"/>
+      <x:c r="W15" s="34"/>
+      <x:c r="X15" s="34"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:M1"/>
-    <x:mergeCell ref="A2:M2"/>
+    <x:mergeCell ref="A1:X1"/>
+    <x:mergeCell ref="A2:X2"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="L5:L15">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="冲突"/>

</xml_diff>